<commit_message>
Update data package at: 2026-09-21T14:43:26Z
</commit_message>
<xml_diff>
--- a/data-raw/desc_fontes_de_recursos.xlsx
+++ b/data-raw/desc_fontes_de_recursos.xlsx
@@ -994,7 +994,7 @@
     <col min="3" max="3" style="7" width="61.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -1038,7 +1038,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1060,7 +1060,7 @@
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1071,7 +1071,7 @@
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1082,7 +1082,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1104,7 +1104,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1126,7 +1126,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1137,7 +1137,7 @@
         <v>26</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>28</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1159,7 +1159,7 @@
         <v>30</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1170,7 +1170,7 @@
         <v>32</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1181,7 +1181,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1192,7 +1192,7 @@
         <v>36</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1203,7 +1203,7 @@
         <v>38</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1357,7 +1357,7 @@
         <v>66</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -1368,7 +1368,7 @@
         <v>68</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -1379,7 +1379,7 @@
         <v>70</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -1390,7 +1390,7 @@
         <v>72</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -1401,7 +1401,7 @@
         <v>74</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -1412,7 +1412,7 @@
         <v>76</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>78</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -1434,7 +1434,7 @@
         <v>80</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -1445,7 +1445,7 @@
         <v>82</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="C42" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>85</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -1476,7 +1476,7 @@
         <v>85</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -1487,7 +1487,7 @@
         <v>88</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
       <c r="A46" s="3">
         <v>45</v>
       </c>
@@ -1498,7 +1498,7 @@
         <v>90</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
       <c r="A47" s="3">
         <v>46</v>
       </c>
@@ -1509,7 +1509,7 @@
         <v>90</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
       <c r="A48" s="3">
         <v>47</v>
       </c>
@@ -1520,7 +1520,7 @@
         <v>93</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
       <c r="A49" s="3">
         <v>48</v>
       </c>
@@ -1531,7 +1531,7 @@
         <v>95</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
       <c r="A50" s="3">
         <v>49</v>
       </c>
@@ -1542,7 +1542,7 @@
         <v>97</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
       <c r="A51" s="3">
         <v>50</v>
       </c>

</xml_diff>